<commit_message>
Audit Trail report: restrict to General Ledger and fix testing issues
- Data model now covers General Ledger only (batch, journal, line field
  changes, reversals, deletions, copies); other modules removed from the SQL
- Transaction ID is the journal name; batch name no longer shown
- Journal action log limited to Copy (Created/Updated events removed)
- Transaction status read from the MJE_BATCH_STATUS lookup
- Coverage sheet removed from the Excel layout
- Add Proof.sql (why AR, receipts, statements, requisitions and payments
  cannot be audited) and PO_Investigation.sql
- Update analysis document, field mapping and discovery queries

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Oracle Fusion Audit Trail Report for Mudad/02_Field_Mapping.xlsx
+++ b/Oracle Fusion Audit Trail Report for Mudad/02_Field_Mapping.xlsx
@@ -61,11 +61,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
@@ -77,6 +72,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -579,7 +579,7 @@
         <v>79</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0</v>
@@ -591,7 +591,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -659,19 +659,19 @@
         <v>54</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>13</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -745,13 +745,13 @@
         <v>0</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>54</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -825,13 +825,13 @@
         <v>0</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>14</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -862,16 +862,16 @@
         <v>1</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>3</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -899,19 +899,19 @@
         <v>23</v>
       </c>
       <c r="D10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="F10" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>1</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -975,19 +975,19 @@
         <v>375</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="F12" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>131</v>
+      </c>
+      <c r="H12" s="3" t="n">
         <v>11</v>
-      </c>
-      <c r="G12" s="3" t="n">
-        <v>125</v>
-      </c>
-      <c r="H12" s="3" t="n">
-        <v>10</v>
       </c>
       <c r="I12" s="3" t="inlineStr"/>
       <c r="J12" s="3" t="inlineStr"/>
@@ -2436,9 +2436,9 @@
           <t>PO-CO - Purchase order change-order history (PO_VERSIONS + PO_*_ARCHIVE_ALL)</t>
         </is>
       </c>
-      <c r="P17" s="5" t="inlineStr">
-        <is>
-          <t>To confirm</t>
+      <c r="P17" s="4" t="inlineStr">
+        <is>
+          <t>Capturable</t>
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr">
@@ -2453,7 +2453,7 @@
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>Not a standard Fusion PO header field; the 'Additional Information' region is normally a descriptive flexfield. Confirm the DFF context/segment. Captured by the same archive comparison once the DFF segment is confirmed.</t>
+          <t>Not a standard Fusion PO header field; the 'Additional Information' region is normally a descriptive flexfield. Confirm the DFF context/segment. Tracked as 'Additional Information &gt; Attribute n' (all 20 header flexfield fields). The attribute number for Payment Type will be renamed once known.</t>
         </is>
       </c>
     </row>
@@ -2523,9 +2523,9 @@
           <t>PO-CO - Purchase order change-order history (PO_VERSIONS + PO_*_ARCHIVE_ALL)</t>
         </is>
       </c>
-      <c r="P18" s="5" t="inlineStr">
-        <is>
-          <t>To confirm</t>
+      <c r="P18" s="4" t="inlineStr">
+        <is>
+          <t>Capturable</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
@@ -2540,7 +2540,7 @@
       </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
-          <t>Not a standard Fusion PO header field; the 'Additional Information' region is normally a descriptive flexfield. Confirm the DFF context/segment. Captured by the same archive comparison once the DFF segment is confirmed.</t>
+          <t>Not a standard Fusion PO header field; the 'Additional Information' region is normally a descriptive flexfield. Confirm the DFF context/segment. Tracked as 'Additional Information &gt; Attribute n' (all 20 header flexfield fields). The attribute number for Payment Status will be renamed once known.</t>
         </is>
       </c>
     </row>
@@ -7590,7 +7590,7 @@
           <t>ATT - Attachment metadata (FND_ATTACHED_DOCUMENTS + FND_DOCUMENTS_TL)</t>
         </is>
       </c>
-      <c r="P75" s="6" t="inlineStr">
+      <c r="P75" s="5" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -8112,7 +8112,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P81" s="7" t="inlineStr">
+      <c r="P81" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -8199,7 +8199,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P82" s="7" t="inlineStr">
+      <c r="P82" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -8286,7 +8286,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P83" s="7" t="inlineStr">
+      <c r="P83" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -8373,7 +8373,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P84" s="7" t="inlineStr">
+      <c r="P84" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -8460,7 +8460,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P85" s="7" t="inlineStr">
+      <c r="P85" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -8547,7 +8547,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P86" s="7" t="inlineStr">
+      <c r="P86" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -8634,7 +8634,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P87" s="7" t="inlineStr">
+      <c r="P87" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -8721,7 +8721,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P88" s="7" t="inlineStr">
+      <c r="P88" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -8808,7 +8808,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P89" s="7" t="inlineStr">
+      <c r="P89" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -8895,7 +8895,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P90" s="7" t="inlineStr">
+      <c r="P90" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -8982,7 +8982,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P91" s="7" t="inlineStr">
+      <c r="P91" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -9069,7 +9069,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P92" s="7" t="inlineStr">
+      <c r="P92" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -9156,7 +9156,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P93" s="7" t="inlineStr">
+      <c r="P93" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -9243,7 +9243,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P94" s="7" t="inlineStr">
+      <c r="P94" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -9330,7 +9330,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P95" s="7" t="inlineStr">
+      <c r="P95" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -9417,7 +9417,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P96" s="7" t="inlineStr">
+      <c r="P96" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -9504,7 +9504,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P97" s="7" t="inlineStr">
+      <c r="P97" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -9591,7 +9591,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P98" s="7" t="inlineStr">
+      <c r="P98" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -9678,7 +9678,7 @@
           <t>ATT - Attachment metadata (FND_ATTACHED_DOCUMENTS + FND_DOCUMENTS_TL)</t>
         </is>
       </c>
-      <c r="P99" s="6" t="inlineStr">
+      <c r="P99" s="5" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -9765,7 +9765,7 @@
           <t>ATT - Attachment metadata (FND_ATTACHED_DOCUMENTS + FND_DOCUMENTS_TL)</t>
         </is>
       </c>
-      <c r="P100" s="6" t="inlineStr">
+      <c r="P100" s="5" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -9852,7 +9852,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P101" s="8" t="inlineStr">
+      <c r="P101" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -9939,7 +9939,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P102" s="8" t="inlineStr">
+      <c r="P102" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -10026,7 +10026,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P103" s="8" t="inlineStr">
+      <c r="P103" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -10113,7 +10113,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P104" s="8" t="inlineStr">
+      <c r="P104" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -10200,7 +10200,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P105" s="8" t="inlineStr">
+      <c r="P105" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -10287,7 +10287,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P106" s="8" t="inlineStr">
+      <c r="P106" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -10374,7 +10374,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P107" s="8" t="inlineStr">
+      <c r="P107" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -10461,7 +10461,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P108" s="8" t="inlineStr">
+      <c r="P108" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -10548,7 +10548,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P109" s="8" t="inlineStr">
+      <c r="P109" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -10635,7 +10635,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P110" s="8" t="inlineStr">
+      <c r="P110" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -10722,9 +10722,9 @@
           <t>ATT - Attachment metadata (FND_ATTACHED_DOCUMENTS + FND_DOCUMENTS_TL)</t>
         </is>
       </c>
-      <c r="P111" s="6" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="P111" s="8" t="inlineStr">
+        <is>
+          <t>To confirm</t>
         </is>
       </c>
       <c r="Q111" s="2" t="inlineStr">
@@ -10734,12 +10734,12 @@
       </c>
       <c r="R111" s="2" t="inlineStr">
         <is>
-          <t>Additions: new value only. Deletions are not recorded.</t>
+          <t>Additions only: no old value. A deleted attachment leaves no row.</t>
         </is>
       </c>
       <c r="S111" s="2" t="inlineStr">
         <is>
-          <t>Deletion of an attachment can only be captured if attachment auditing is available (not confirmed).</t>
+          <t>Built for PO, requisition and payment attachments. Invoice attachments are added once one exists in TEST, so the attachment type name can be read.</t>
         </is>
       </c>
     </row>
@@ -10813,7 +10813,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P112" s="8" t="inlineStr">
+      <c r="P112" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -10904,7 +10904,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P113" s="8" t="inlineStr">
+      <c r="P113" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -10995,7 +10995,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P114" s="8" t="inlineStr">
+      <c r="P114" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -11086,7 +11086,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P115" s="8" t="inlineStr">
+      <c r="P115" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -11181,7 +11181,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P116" s="8" t="inlineStr">
+      <c r="P116" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -11272,7 +11272,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P117" s="8" t="inlineStr">
+      <c r="P117" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -11363,7 +11363,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P118" s="8" t="inlineStr">
+      <c r="P118" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -11454,7 +11454,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P119" s="8" t="inlineStr">
+      <c r="P119" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -11549,7 +11549,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P120" s="8" t="inlineStr">
+      <c r="P120" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -11644,7 +11644,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P121" s="8" t="inlineStr">
+      <c r="P121" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -11735,7 +11735,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P122" s="8" t="inlineStr">
+      <c r="P122" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -11830,7 +11830,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P123" s="8" t="inlineStr">
+      <c r="P123" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -11925,7 +11925,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P124" s="8" t="inlineStr">
+      <c r="P124" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -12020,7 +12020,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P125" s="8" t="inlineStr">
+      <c r="P125" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -12115,7 +12115,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P126" s="8" t="inlineStr">
+      <c r="P126" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -12210,7 +12210,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P127" s="8" t="inlineStr">
+      <c r="P127" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -12305,7 +12305,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P128" s="8" t="inlineStr">
+      <c r="P128" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -12400,7 +12400,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P129" s="8" t="inlineStr">
+      <c r="P129" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -12495,7 +12495,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P130" s="8" t="inlineStr">
+      <c r="P130" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -12590,7 +12590,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P131" s="8" t="inlineStr">
+      <c r="P131" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -12685,7 +12685,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P132" s="8" t="inlineStr">
+      <c r="P132" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -12776,7 +12776,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P133" s="8" t="inlineStr">
+      <c r="P133" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -12867,7 +12867,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P134" s="8" t="inlineStr">
+      <c r="P134" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -12958,7 +12958,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P135" s="8" t="inlineStr">
+      <c r="P135" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -13049,7 +13049,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P136" s="8" t="inlineStr">
+      <c r="P136" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -13140,7 +13140,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P137" s="8" t="inlineStr">
+      <c r="P137" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -13235,7 +13235,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P138" s="8" t="inlineStr">
+      <c r="P138" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -13330,7 +13330,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P139" s="8" t="inlineStr">
+      <c r="P139" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -13425,7 +13425,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P140" s="8" t="inlineStr">
+      <c r="P140" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -13520,7 +13520,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P141" s="8" t="inlineStr">
+      <c r="P141" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -13615,7 +13615,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P142" s="8" t="inlineStr">
+      <c r="P142" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -13632,7 +13632,7 @@
       </c>
       <c r="S142" s="2" t="inlineStr">
         <is>
-          <t>Audit object: Payables &gt; Invoice Lines (audit table AP_INVOICE_LINES_ALL_).</t>
+          <t>Start Date (DEF_ACCTG_START_DATE): enabled in TEST on 18 Oct 2026.</t>
         </is>
       </c>
     </row>
@@ -13710,7 +13710,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P143" s="8" t="inlineStr">
+      <c r="P143" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -13805,7 +13805,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P144" s="8" t="inlineStr">
+      <c r="P144" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -13822,7 +13822,7 @@
       </c>
       <c r="S144" s="2" t="inlineStr">
         <is>
-          <t>Audit object: Payables &gt; Invoice Lines (audit table AP_INVOICE_LINES_ALL_).</t>
+          <t>Accrual Account (DEF_ACCTG_ACCRUAL_CCID): enabled in TEST on 18 Oct 2026.</t>
         </is>
       </c>
     </row>
@@ -13900,9 +13900,9 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P145" s="8" t="inlineStr">
-        <is>
-          <t>Capturable after setup</t>
+      <c r="P145" s="6" t="inlineStr">
+        <is>
+          <t>Not capturable</t>
         </is>
       </c>
       <c r="Q145" s="2" t="inlineStr">
@@ -13917,7 +13917,7 @@
       </c>
       <c r="S145" s="2" t="inlineStr">
         <is>
-          <t>Assumed to be Mudad chart-of-accounts segments of the distribution combination. Confirm the segment names; if Region is a descriptive flexfield instead, say so. Audit object: Payables &gt; Invoice Lines (audit table AP_INVOICE_LINES_ALL_). Field meaning or column still to confirm.</t>
+          <t>Assumed to be Mudad chart-of-accounts segments of the distribution combination. Confirm the segment names; if Region is a descriptive flexfield instead, say so. Income Tax Region: Not offered on the audit setup page for this object (checked in Mudad TEST, 18 Oct 2026), so Fusion cannot audit it.</t>
         </is>
       </c>
     </row>
@@ -13991,7 +13991,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P146" s="8" t="inlineStr">
+      <c r="P146" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -14086,7 +14086,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P147" s="8" t="inlineStr">
+      <c r="P147" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -14181,7 +14181,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P148" s="8" t="inlineStr">
+      <c r="P148" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -14276,7 +14276,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P149" s="8" t="inlineStr">
+      <c r="P149" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -14371,7 +14371,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P150" s="8" t="inlineStr">
+      <c r="P150" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -14466,7 +14466,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P151" s="8" t="inlineStr">
+      <c r="P151" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -14483,7 +14483,7 @@
       </c>
       <c r="S151" s="2" t="inlineStr">
         <is>
-          <t>Audit object: Payables &gt; Invoice Lines (audit table AP_INVOICE_LINES_ALL_).</t>
+          <t>Asset Book (ASSET_BOOK_TYPE_CODE): enabled in TEST on 18 Oct 2026.</t>
         </is>
       </c>
     </row>
@@ -14561,9 +14561,9 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P152" s="8" t="inlineStr">
-        <is>
-          <t>Capturable after setup</t>
+      <c r="P152" s="6" t="inlineStr">
+        <is>
+          <t>Not capturable</t>
         </is>
       </c>
       <c r="Q152" s="2" t="inlineStr">
@@ -14578,7 +14578,7 @@
       </c>
       <c r="S152" s="2" t="inlineStr">
         <is>
-          <t>Audit object: Payables &gt; Invoice Lines (audit table AP_INVOICE_LINES_ALL_).</t>
+          <t>Asset Category: Not offered on the audit setup page for this object (checked in Mudad TEST, 18 Oct 2026), so Fusion cannot audit it.</t>
         </is>
       </c>
     </row>
@@ -14652,9 +14652,9 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P153" s="8" t="inlineStr">
-        <is>
-          <t>Capturable after setup</t>
+      <c r="P153" s="6" t="inlineStr">
+        <is>
+          <t>Not capturable</t>
         </is>
       </c>
       <c r="Q153" s="2" t="inlineStr">
@@ -14669,7 +14669,7 @@
       </c>
       <c r="S153" s="2" t="inlineStr">
         <is>
-          <t>Audit object: Payables &gt; Invoice Lines (audit table AP_INVOICE_LINES_ALL_). Field meaning or column still to confirm.</t>
+          <t>Correction Type: Not offered on the audit setup page for this object (checked in Mudad TEST, 18 Oct 2026), so Fusion cannot audit it.</t>
         </is>
       </c>
     </row>
@@ -14743,7 +14743,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P154" s="8" t="inlineStr">
+      <c r="P154" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -14834,7 +14834,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P155" s="8" t="inlineStr">
+      <c r="P155" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -14923,7 +14923,7 @@
       </c>
       <c r="P156" s="6" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Not capturable</t>
         </is>
       </c>
       <c r="Q156" s="2" t="inlineStr">
@@ -14938,7 +14938,7 @@
       </c>
       <c r="S156" s="2" t="inlineStr">
         <is>
-          <t>Tax lines are rows of AP_INVOICE_LINES_ALL, but tax recalculated by the application is not audited (only user-initiated updates are).</t>
+          <t>Tax Rate Name: Not offered on the audit setup page for this object (checked in Mudad TEST, 18 Oct 2026), so Fusion cannot audit it.</t>
         </is>
       </c>
     </row>
@@ -15012,7 +15012,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P157" s="8" t="inlineStr">
+      <c r="P157" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -15103,7 +15103,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P158" s="8" t="inlineStr">
+      <c r="P158" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -15194,7 +15194,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P159" s="8" t="inlineStr">
+      <c r="P159" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -15285,7 +15285,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P160" s="8" t="inlineStr">
+      <c r="P160" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -15376,7 +15376,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P161" s="8" t="inlineStr">
+      <c r="P161" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -15467,7 +15467,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P162" s="8" t="inlineStr">
+      <c r="P162" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -15558,7 +15558,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P163" s="8" t="inlineStr">
+      <c r="P163" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -15649,7 +15649,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P164" s="8" t="inlineStr">
+      <c r="P164" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -15740,7 +15740,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P165" s="8" t="inlineStr">
+      <c r="P165" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -15827,7 +15827,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P166" s="8" t="inlineStr">
+      <c r="P166" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -15914,7 +15914,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P167" s="8" t="inlineStr">
+      <c r="P167" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -16001,7 +16001,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P168" s="8" t="inlineStr">
+      <c r="P168" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -16088,7 +16088,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P169" s="8" t="inlineStr">
+      <c r="P169" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -16175,7 +16175,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P170" s="8" t="inlineStr">
+      <c r="P170" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -16262,7 +16262,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P171" s="6" t="inlineStr">
+      <c r="P171" s="5" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -16349,9 +16349,9 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P172" s="8" t="inlineStr">
-        <is>
-          <t>Capturable after setup</t>
+      <c r="P172" s="5" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="Q172" s="2" t="inlineStr">
@@ -16366,7 +16366,7 @@
       </c>
       <c r="S172" s="2" t="inlineStr">
         <is>
-          <t>Installment-level hold (hold flag on the installment). Audit object: Payables &gt; Invoice Installments (audit table AP_PAYMENT_SCHEDULES_ALL_).</t>
+          <t>Installment-level hold (hold flag on the installment). The installment hold flag is not offered. Only Hold Reason (IBY_HOLD_REASON) is audited, so a placed or released hold shows as a change of hold reason.</t>
         </is>
       </c>
     </row>
@@ -16436,9 +16436,9 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P173" s="8" t="inlineStr">
-        <is>
-          <t>Capturable after setup</t>
+      <c r="P173" s="5" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="Q173" s="2" t="inlineStr">
@@ -16453,7 +16453,7 @@
       </c>
       <c r="S173" s="2" t="inlineStr">
         <is>
-          <t>Installment-level hold (hold flag on the installment). Audit object: Payables &gt; Invoice Installments (audit table AP_PAYMENT_SCHEDULES_ALL_).</t>
+          <t>Installment-level hold (hold flag on the installment). The installment hold flag is not offered. Only Hold Reason (IBY_HOLD_REASON) is audited, so a placed or released hold shows as a change of hold reason.</t>
         </is>
       </c>
     </row>
@@ -16523,9 +16523,9 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P174" s="8" t="inlineStr">
-        <is>
-          <t>Capturable after setup</t>
+      <c r="P174" s="6" t="inlineStr">
+        <is>
+          <t>Not capturable</t>
         </is>
       </c>
       <c r="Q174" s="2" t="inlineStr">
@@ -16540,7 +16540,7 @@
       </c>
       <c r="S174" s="2" t="inlineStr">
         <is>
-          <t>Audit object: Payables &gt; Invoice Installments (audit table AP_PAYMENT_SCHEDULES_ALL_).</t>
+          <t>Discount Date: Not offered on the audit setup page for this object (checked in Mudad TEST, 18 Oct 2026), so Fusion cannot audit it. (Only Discount APR / Discount Campaign are offered, which belong to dynamic discounting.)</t>
         </is>
       </c>
     </row>
@@ -16610,9 +16610,9 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P175" s="8" t="inlineStr">
-        <is>
-          <t>Capturable after setup</t>
+      <c r="P175" s="6" t="inlineStr">
+        <is>
+          <t>Not capturable</t>
         </is>
       </c>
       <c r="Q175" s="2" t="inlineStr">
@@ -16627,7 +16627,7 @@
       </c>
       <c r="S175" s="2" t="inlineStr">
         <is>
-          <t>Audit object: Payables &gt; Invoice Installments (audit table AP_PAYMENT_SCHEDULES_ALL_).</t>
+          <t>Discount amount: Not offered on the audit setup page for this object (checked in Mudad TEST, 18 Oct 2026), so Fusion cannot audit it.</t>
         </is>
       </c>
     </row>
@@ -16697,7 +16697,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P176" s="8" t="inlineStr">
+      <c r="P176" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -16784,7 +16784,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P177" s="8" t="inlineStr">
+      <c r="P177" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -16871,7 +16871,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P178" s="8" t="inlineStr">
+      <c r="P178" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -17045,7 +17045,7 @@
           <t>ATT - Attachment metadata (FND_ATTACHED_DOCUMENTS + FND_DOCUMENTS_TL)</t>
         </is>
       </c>
-      <c r="P180" s="6" t="inlineStr">
+      <c r="P180" s="5" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -17132,7 +17132,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P181" s="7" t="inlineStr">
+      <c r="P181" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -17219,7 +17219,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P182" s="7" t="inlineStr">
+      <c r="P182" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -17306,7 +17306,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P183" s="7" t="inlineStr">
+      <c r="P183" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -17393,7 +17393,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P184" s="7" t="inlineStr">
+      <c r="P184" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -17480,7 +17480,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P185" s="7" t="inlineStr">
+      <c r="P185" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -17567,7 +17567,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P186" s="7" t="inlineStr">
+      <c r="P186" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -17654,7 +17654,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P187" s="7" t="inlineStr">
+      <c r="P187" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -17741,7 +17741,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P188" s="7" t="inlineStr">
+      <c r="P188" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -17828,7 +17828,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P189" s="7" t="inlineStr">
+      <c r="P189" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -17915,7 +17915,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P190" s="7" t="inlineStr">
+      <c r="P190" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -18006,7 +18006,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P191" s="7" t="inlineStr">
+      <c r="P191" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -18093,7 +18093,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P192" s="7" t="inlineStr">
+      <c r="P192" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -18180,7 +18180,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P193" s="7" t="inlineStr">
+      <c r="P193" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -18267,7 +18267,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P194" s="7" t="inlineStr">
+      <c r="P194" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -18354,7 +18354,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P195" s="7" t="inlineStr">
+      <c r="P195" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -18441,7 +18441,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P196" s="7" t="inlineStr">
+      <c r="P196" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -18528,7 +18528,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P197" s="7" t="inlineStr">
+      <c r="P197" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -18615,7 +18615,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P198" s="7" t="inlineStr">
+      <c r="P198" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -18702,7 +18702,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P199" s="7" t="inlineStr">
+      <c r="P199" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -18789,7 +18789,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P200" s="7" t="inlineStr">
+      <c r="P200" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -18876,7 +18876,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P201" s="7" t="inlineStr">
+      <c r="P201" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -18963,7 +18963,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P202" s="7" t="inlineStr">
+      <c r="P202" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -19050,7 +19050,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P203" s="7" t="inlineStr">
+      <c r="P203" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -19141,7 +19141,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P204" s="7" t="inlineStr">
+      <c r="P204" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -19228,7 +19228,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P205" s="7" t="inlineStr">
+      <c r="P205" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -19315,7 +19315,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P206" s="7" t="inlineStr">
+      <c r="P206" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -19406,7 +19406,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P207" s="7" t="inlineStr">
+      <c r="P207" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -19497,7 +19497,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P208" s="7" t="inlineStr">
+      <c r="P208" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -19588,7 +19588,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P209" s="7" t="inlineStr">
+      <c r="P209" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -19679,7 +19679,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P210" s="7" t="inlineStr">
+      <c r="P210" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -19770,7 +19770,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P211" s="7" t="inlineStr">
+      <c r="P211" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -19861,7 +19861,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P212" s="7" t="inlineStr">
+      <c r="P212" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -19952,7 +19952,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P213" s="7" t="inlineStr">
+      <c r="P213" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -20039,7 +20039,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P214" s="7" t="inlineStr">
+      <c r="P214" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -20126,7 +20126,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P215" s="7" t="inlineStr">
+      <c r="P215" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -20213,7 +20213,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P216" s="7" t="inlineStr">
+      <c r="P216" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -20300,7 +20300,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P217" s="7" t="inlineStr">
+      <c r="P217" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -20387,7 +20387,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P218" s="7" t="inlineStr">
+      <c r="P218" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -20474,7 +20474,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P219" s="7" t="inlineStr">
+      <c r="P219" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -20561,9 +20561,9 @@
           <t>ATT - Attachment metadata (FND_ATTACHED_DOCUMENTS + FND_DOCUMENTS_TL)</t>
         </is>
       </c>
-      <c r="P220" s="6" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="P220" s="8" t="inlineStr">
+        <is>
+          <t>To confirm</t>
         </is>
       </c>
       <c r="Q220" s="2" t="inlineStr">
@@ -20573,12 +20573,12 @@
       </c>
       <c r="R220" s="2" t="inlineStr">
         <is>
-          <t>Additions: new value only. Deletions are not recorded.</t>
+          <t>Additions only: no old value. A deleted attachment leaves no row.</t>
         </is>
       </c>
       <c r="S220" s="2" t="inlineStr">
         <is>
-          <t>Deletion of an attachment can only be captured if attachment auditing is available (not confirmed).</t>
+          <t>As for invoice attachments: added once a receipt attachment exists in TEST.</t>
         </is>
       </c>
     </row>
@@ -20648,7 +20648,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P221" s="7" t="inlineStr">
+      <c r="P221" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -20735,7 +20735,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P222" s="7" t="inlineStr">
+      <c r="P222" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -20822,7 +20822,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P223" s="7" t="inlineStr">
+      <c r="P223" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -20909,7 +20909,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P224" s="7" t="inlineStr">
+      <c r="P224" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -20996,7 +20996,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P225" s="7" t="inlineStr">
+      <c r="P225" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -21083,7 +21083,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P226" s="7" t="inlineStr">
+      <c r="P226" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -21170,7 +21170,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P227" s="7" t="inlineStr">
+      <c r="P227" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -21257,7 +21257,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P228" s="7" t="inlineStr">
+      <c r="P228" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -21344,7 +21344,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P229" s="7" t="inlineStr">
+      <c r="P229" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -21431,7 +21431,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P230" s="7" t="inlineStr">
+      <c r="P230" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -21518,7 +21518,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P231" s="7" t="inlineStr">
+      <c r="P231" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -21605,7 +21605,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P232" s="7" t="inlineStr">
+      <c r="P232" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -22277,7 +22277,7 @@
           <t>AR-APP - Receipt applications (AR_RECEIVABLE_APPLICATIONS_ALL)</t>
         </is>
       </c>
-      <c r="P240" s="5" t="inlineStr">
+      <c r="P240" s="8" t="inlineStr">
         <is>
           <t>To confirm</t>
         </is>
@@ -22364,7 +22364,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P241" s="7" t="inlineStr">
+      <c r="P241" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -22451,7 +22451,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P242" s="7" t="inlineStr">
+      <c r="P242" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -22538,7 +22538,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P243" s="7" t="inlineStr">
+      <c r="P243" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -22625,7 +22625,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P244" s="7" t="inlineStr">
+      <c r="P244" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -22712,7 +22712,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P245" s="7" t="inlineStr">
+      <c r="P245" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -22799,7 +22799,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P246" s="7" t="inlineStr">
+      <c r="P246" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -22886,7 +22886,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P247" s="7" t="inlineStr">
+      <c r="P247" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -22973,9 +22973,9 @@
           <t>ATT - Attachment metadata (FND_ATTACHED_DOCUMENTS + FND_DOCUMENTS_TL)</t>
         </is>
       </c>
-      <c r="P248" s="6" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="P248" s="8" t="inlineStr">
+        <is>
+          <t>To confirm</t>
         </is>
       </c>
       <c r="Q248" s="2" t="inlineStr">
@@ -22985,12 +22985,12 @@
       </c>
       <c r="R248" s="2" t="inlineStr">
         <is>
-          <t>Additions: new value only. Deletions are not recorded.</t>
+          <t>Additions only: no old value. A deleted attachment leaves no row.</t>
         </is>
       </c>
       <c r="S248" s="2" t="inlineStr">
         <is>
-          <t>Deletion of an attachment can only be captured if attachment auditing is available (not confirmed).</t>
+          <t>As for invoice attachments: added once a statement attachment exists in TEST.</t>
         </is>
       </c>
     </row>
@@ -23060,7 +23060,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P249" s="7" t="inlineStr">
+      <c r="P249" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -23147,7 +23147,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P250" s="7" t="inlineStr">
+      <c r="P250" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -23234,7 +23234,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P251" s="7" t="inlineStr">
+      <c r="P251" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -23321,7 +23321,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P252" s="7" t="inlineStr">
+      <c r="P252" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -23408,7 +23408,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P253" s="7" t="inlineStr">
+      <c r="P253" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -23495,7 +23495,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P254" s="7" t="inlineStr">
+      <c r="P254" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -23582,7 +23582,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P255" s="6" t="inlineStr">
+      <c r="P255" s="5" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -23669,7 +23669,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P256" s="7" t="inlineStr">
+      <c r="P256" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -23756,7 +23756,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P257" s="7" t="inlineStr">
+      <c r="P257" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -23843,7 +23843,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P258" s="7" t="inlineStr">
+      <c r="P258" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -23930,7 +23930,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P259" s="7" t="inlineStr">
+      <c r="P259" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -24017,7 +24017,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P260" s="7" t="inlineStr">
+      <c r="P260" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -24104,7 +24104,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P261" s="7" t="inlineStr">
+      <c r="P261" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -24191,7 +24191,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P262" s="7" t="inlineStr">
+      <c r="P262" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -24278,7 +24278,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P263" s="7" t="inlineStr">
+      <c r="P263" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -24365,7 +24365,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P264" s="7" t="inlineStr">
+      <c r="P264" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -24452,7 +24452,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P265" s="7" t="inlineStr">
+      <c r="P265" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -24539,7 +24539,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P266" s="7" t="inlineStr">
+      <c r="P266" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -24626,7 +24626,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P267" s="7" t="inlineStr">
+      <c r="P267" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -24713,7 +24713,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P268" s="7" t="inlineStr">
+      <c r="P268" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -24800,7 +24800,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P269" s="7" t="inlineStr">
+      <c r="P269" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -24887,7 +24887,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P270" s="7" t="inlineStr">
+      <c r="P270" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -24974,7 +24974,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P271" s="7" t="inlineStr">
+      <c r="P271" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -25061,7 +25061,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P272" s="7" t="inlineStr">
+      <c r="P272" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -25148,7 +25148,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P273" s="7" t="inlineStr">
+      <c r="P273" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -25235,7 +25235,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P274" s="7" t="inlineStr">
+      <c r="P274" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -25322,7 +25322,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P275" s="7" t="inlineStr">
+      <c r="P275" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -25409,7 +25409,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P276" s="7" t="inlineStr">
+      <c r="P276" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -25496,7 +25496,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P277" s="7" t="inlineStr">
+      <c r="P277" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -25583,7 +25583,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P278" s="7" t="inlineStr">
+      <c r="P278" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -25670,7 +25670,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P279" s="7" t="inlineStr">
+      <c r="P279" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -25757,7 +25757,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P280" s="7" t="inlineStr">
+      <c r="P280" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -25844,7 +25844,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P281" s="7" t="inlineStr">
+      <c r="P281" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -25931,7 +25931,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P282" s="7" t="inlineStr">
+      <c r="P282" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -26018,7 +26018,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P283" s="7" t="inlineStr">
+      <c r="P283" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -26105,7 +26105,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P284" s="7" t="inlineStr">
+      <c r="P284" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -26192,7 +26192,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P285" s="7" t="inlineStr">
+      <c r="P285" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -26279,7 +26279,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P286" s="7" t="inlineStr">
+      <c r="P286" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -26366,7 +26366,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P287" s="7" t="inlineStr">
+      <c r="P287" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -26453,7 +26453,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P288" s="7" t="inlineStr">
+      <c r="P288" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -26540,7 +26540,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P289" s="7" t="inlineStr">
+      <c r="P289" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -26627,7 +26627,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P290" s="7" t="inlineStr">
+      <c r="P290" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -26714,7 +26714,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P291" s="7" t="inlineStr">
+      <c r="P291" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -26801,7 +26801,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P292" s="7" t="inlineStr">
+      <c r="P292" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -26888,7 +26888,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P293" s="7" t="inlineStr">
+      <c r="P293" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -26975,7 +26975,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P294" s="7" t="inlineStr">
+      <c r="P294" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -27062,7 +27062,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P295" s="7" t="inlineStr">
+      <c r="P295" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -27149,7 +27149,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P296" s="7" t="inlineStr">
+      <c r="P296" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -28549,7 +28549,7 @@
           <t>FA-TRX - Asset transaction history (FA_TRANSACTION_HEADERS + FA_BOOKS / FA_ASSET_HISTORY / FA_DISTRIBUTION_HISTORY / FA_RETIREMENTS)</t>
         </is>
       </c>
-      <c r="P312" s="5" t="inlineStr">
+      <c r="P312" s="8" t="inlineStr">
         <is>
           <t>To confirm</t>
         </is>
@@ -28640,7 +28640,7 @@
           <t>FA-TRX - Asset transaction history (FA_TRANSACTION_HEADERS + FA_BOOKS / FA_ASSET_HISTORY / FA_DISTRIBUTION_HISTORY / FA_RETIREMENTS)</t>
         </is>
       </c>
-      <c r="P313" s="5" t="inlineStr">
+      <c r="P313" s="8" t="inlineStr">
         <is>
           <t>To confirm</t>
         </is>
@@ -28818,7 +28818,7 @@
           <t>FA-TRX - Asset transaction history (FA_TRANSACTION_HEADERS + FA_BOOKS / FA_ASSET_HISTORY / FA_DISTRIBUTION_HISTORY / FA_RETIREMENTS)</t>
         </is>
       </c>
-      <c r="P315" s="5" t="inlineStr">
+      <c r="P315" s="8" t="inlineStr">
         <is>
           <t>To confirm</t>
         </is>
@@ -29846,7 +29846,7 @@
           <t>FA-TRX - Asset transaction history (FA_TRANSACTION_HEADERS + FA_BOOKS / FA_ASSET_HISTORY / FA_DISTRIBUTION_HISTORY / FA_RETIREMENTS)</t>
         </is>
       </c>
-      <c r="P327" s="5" t="inlineStr">
+      <c r="P327" s="8" t="inlineStr">
         <is>
           <t>To confirm</t>
         </is>
@@ -30597,24 +30597,24 @@
           <t>ESS - Scheduled process history</t>
         </is>
       </c>
-      <c r="P336" s="5" t="inlineStr">
-        <is>
-          <t>To confirm</t>
+      <c r="P336" s="4" t="inlineStr">
+        <is>
+          <t>Capturable</t>
         </is>
       </c>
       <c r="Q336" s="2" t="inlineStr">
         <is>
-          <t>To verify in the pod (check C13)</t>
+          <t>Verified in Mudad TEST (ESS_REQUEST_HISTORY readable)</t>
         </is>
       </c>
       <c r="R336" s="2" t="inlineStr">
         <is>
-          <t>No field values.</t>
+          <t>Process run: who, when, status.</t>
         </is>
       </c>
       <c r="S336" s="2" t="inlineStr">
         <is>
-          <t>Process, not a field change. Can only be logged as 'scheduled process submitted by / at'. Process event, not a change to an asset (Q13).</t>
+          <t>Process, not a field change. Can only be logged as 'scheduled process submitted by / at'. From the scheduled-process history (ESS_REQUEST_HISTORY): Calculate Depreciation runs.</t>
         </is>
       </c>
     </row>
@@ -30684,24 +30684,24 @@
           <t>ESS - Scheduled process history</t>
         </is>
       </c>
-      <c r="P337" s="5" t="inlineStr">
-        <is>
-          <t>To confirm</t>
+      <c r="P337" s="4" t="inlineStr">
+        <is>
+          <t>Capturable</t>
         </is>
       </c>
       <c r="Q337" s="2" t="inlineStr">
         <is>
-          <t>To verify in the pod (check C13)</t>
+          <t>Verified in Mudad TEST (ESS_REQUEST_HISTORY readable)</t>
         </is>
       </c>
       <c r="R337" s="2" t="inlineStr">
         <is>
-          <t>No field values.</t>
+          <t>Process run: who, when, status.</t>
         </is>
       </c>
       <c r="S337" s="2" t="inlineStr">
         <is>
-          <t>Process, not a field change. Can only be logged as 'scheduled process submitted by / at'. Process event, not a change to an asset (Q13).</t>
+          <t>Process, not a field change. Can only be logged as 'scheduled process submitted by / at'. From the scheduled-process history (ESS_REQUEST_HISTORY): Close Period runs.</t>
         </is>
       </c>
     </row>
@@ -30858,7 +30858,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P339" s="8" t="inlineStr">
+      <c r="P339" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -30949,7 +30949,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P340" s="7" t="inlineStr">
+      <c r="P340" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -31040,7 +31040,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P341" s="8" t="inlineStr">
+      <c r="P341" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -31131,7 +31131,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P342" s="8" t="inlineStr">
+      <c r="P342" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -31222,7 +31222,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P343" s="8" t="inlineStr">
+      <c r="P343" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -31313,7 +31313,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P344" s="8" t="inlineStr">
+      <c r="P344" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -31404,7 +31404,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P345" s="8" t="inlineStr">
+      <c r="P345" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -31495,7 +31495,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P346" s="8" t="inlineStr">
+      <c r="P346" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -31586,7 +31586,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P347" s="8" t="inlineStr">
+      <c r="P347" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -31677,7 +31677,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P348" s="8" t="inlineStr">
+      <c r="P348" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -31768,7 +31768,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P349" s="8" t="inlineStr">
+      <c r="P349" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -31859,7 +31859,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P350" s="8" t="inlineStr">
+      <c r="P350" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -31950,7 +31950,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P351" s="8" t="inlineStr">
+      <c r="P351" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -32041,7 +32041,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P352" s="8" t="inlineStr">
+      <c r="P352" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -32132,9 +32132,9 @@
           <t>ATT - Attachment metadata (FND_ATTACHED_DOCUMENTS + FND_DOCUMENTS_TL)</t>
         </is>
       </c>
-      <c r="P353" s="6" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="P353" s="8" t="inlineStr">
+        <is>
+          <t>To confirm</t>
         </is>
       </c>
       <c r="Q353" s="2" t="inlineStr">
@@ -32144,12 +32144,12 @@
       </c>
       <c r="R353" s="2" t="inlineStr">
         <is>
-          <t>Additions: new value only. Deletions are not recorded.</t>
+          <t>Additions only: no old value. A deleted attachment leaves no row.</t>
         </is>
       </c>
       <c r="S353" s="2" t="inlineStr">
         <is>
-          <t>Deletion of an attachment can only be captured if attachment auditing is available (not confirmed).</t>
+          <t>As for invoice attachments: added once an asset attachment exists in TEST.</t>
         </is>
       </c>
     </row>
@@ -32219,7 +32219,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P354" s="8" t="inlineStr">
+      <c r="P354" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -32306,7 +32306,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P355" s="8" t="inlineStr">
+      <c r="P355" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -32393,9 +32393,9 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P356" s="8" t="inlineStr">
-        <is>
-          <t>Capturable after setup</t>
+      <c r="P356" s="5" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="Q356" s="2" t="inlineStr">
@@ -32410,7 +32410,7 @@
       </c>
       <c r="S356" s="2" t="inlineStr">
         <is>
-          <t>Audit object: General Ledger &gt; Journals &gt; Journal Batch (audit table GL_JE_BATCHES_). Audit table documented by Oracle; confirm the attribute is offered on the setup page.</t>
+          <t>Batch Accounting Period is not offered on the audit setup page (checked in TEST, 18 Oct 2026). A period change still shows through the audited journal Accounting Date (GL_JE_HEADERS.DEFAULT_EFFECTIVE_DATE).</t>
         </is>
       </c>
     </row>
@@ -32477,27 +32477,27 @@
       </c>
       <c r="O357" s="2" t="inlineStr">
         <is>
-          <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
+          <t>ATT - Attachment metadata (FND_ATTACHED_DOCUMENTS + FND_DOCUMENTS_TL)</t>
         </is>
       </c>
       <c r="P357" s="8" t="inlineStr">
         <is>
-          <t>Capturable after setup</t>
+          <t>To confirm</t>
         </is>
       </c>
       <c r="Q357" s="2" t="inlineStr">
         <is>
-          <t>Oracle doc (26D)</t>
+          <t>Oracle doc (26D oedma); used by the P2P Dashboard</t>
         </is>
       </c>
       <c r="R357" s="2" t="inlineStr">
         <is>
-          <t>Yes - attachment added / updated / deleted.</t>
+          <t>Additions only: no old value. A deleted attachment leaves no row.</t>
         </is>
       </c>
       <c r="S357" s="2" t="inlineStr">
         <is>
-          <t>Journal attachment audit (General Ledger &gt; Journals, available since 24A): add, update, delete and download of attachments added in the UI.</t>
+          <t>As for invoice attachments: added once a journal attachment exists in TEST.</t>
         </is>
       </c>
     </row>
@@ -32567,7 +32567,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P358" s="8" t="inlineStr">
+      <c r="P358" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -32654,7 +32654,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P359" s="8" t="inlineStr">
+      <c r="P359" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -32741,7 +32741,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P360" s="8" t="inlineStr">
+      <c r="P360" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -32828,7 +32828,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P361" s="8" t="inlineStr">
+      <c r="P361" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -32915,7 +32915,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P362" s="8" t="inlineStr">
+      <c r="P362" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -32999,27 +32999,27 @@
       </c>
       <c r="O363" s="2" t="inlineStr">
         <is>
-          <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
+          <t>ATT - Attachment metadata (FND_ATTACHED_DOCUMENTS + FND_DOCUMENTS_TL)</t>
         </is>
       </c>
       <c r="P363" s="8" t="inlineStr">
         <is>
-          <t>Capturable after setup</t>
+          <t>To confirm</t>
         </is>
       </c>
       <c r="Q363" s="2" t="inlineStr">
         <is>
-          <t>Oracle doc (26D)</t>
+          <t>Oracle doc (26D oedma); used by the P2P Dashboard</t>
         </is>
       </c>
       <c r="R363" s="2" t="inlineStr">
         <is>
-          <t>Yes - attachment added / updated / deleted.</t>
+          <t>Additions only: no old value. A deleted attachment leaves no row.</t>
         </is>
       </c>
       <c r="S363" s="2" t="inlineStr">
         <is>
-          <t>Journal attachment audit (General Ledger &gt; Journals, available since 24A): add, update, delete and download of attachments added in the UI.</t>
+          <t>As for invoice attachments: added once a journal attachment exists in TEST.</t>
         </is>
       </c>
     </row>
@@ -33089,7 +33089,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P364" s="8" t="inlineStr">
+      <c r="P364" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -33176,7 +33176,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P365" s="8" t="inlineStr">
+      <c r="P365" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -33263,7 +33263,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P366" s="8" t="inlineStr">
+      <c r="P366" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -33350,7 +33350,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P367" s="8" t="inlineStr">
+      <c r="P367" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -33437,7 +33437,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P368" s="8" t="inlineStr">
+      <c r="P368" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -33524,7 +33524,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P369" s="8" t="inlineStr">
+      <c r="P369" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -33611,7 +33611,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P370" s="8" t="inlineStr">
+      <c r="P370" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -33698,7 +33698,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P371" s="8" t="inlineStr">
+      <c r="P371" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -33785,7 +33785,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P372" s="8" t="inlineStr">
+      <c r="P372" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -33955,7 +33955,7 @@
           <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
         </is>
       </c>
-      <c r="P374" s="8" t="inlineStr">
+      <c r="P374" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -34039,27 +34039,27 @@
       </c>
       <c r="O375" s="2" t="inlineStr">
         <is>
-          <t>AUDIT - Fusion audit policy history (&lt;base table&gt;_ audit tables)</t>
-        </is>
-      </c>
-      <c r="P375" s="5" t="inlineStr">
-        <is>
-          <t>To confirm</t>
+          <t>GL-REV - Journal reversal link (GL_JE_HEADERS)</t>
+        </is>
+      </c>
+      <c r="P375" s="4" t="inlineStr">
+        <is>
+          <t>Capturable</t>
         </is>
       </c>
       <c r="Q375" s="2" t="inlineStr">
         <is>
-          <t>Oracle doc (26D)</t>
+          <t>Oracle doc (26D oedmf)</t>
         </is>
       </c>
       <c r="R375" s="2" t="inlineStr">
         <is>
-          <t>Yes - previous audit row for the same key. The first change after auditing is switched on may have no earlier row (validation test V-01).</t>
+          <t>Copied journal name.</t>
         </is>
       </c>
       <c r="S375" s="2" t="inlineStr">
         <is>
-          <t>A copied batch is a new batch (its CREATED_BY / CREATION_DATE are recorded). Whether the source batch is recorded depends on GL_JE_ACTION_LOG content (C11).</t>
+          <t>From the journal action log (GL_JE_ACTION_LOG, ACTION_CODE / TARGET_JE_HEADER_ID).</t>
         </is>
       </c>
     </row>
@@ -34129,7 +34129,7 @@
           <t>NONE - No supported source</t>
         </is>
       </c>
-      <c r="P376" s="7" t="inlineStr">
+      <c r="P376" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -34535,7 +34535,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>To verify in the pod (check C13)</t>
+          <t>Verified in Mudad TEST (ESS_REQUEST_HISTORY readable)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -34625,7 +34625,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Capturable after setup</t>
         </is>
@@ -34637,7 +34637,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -34649,7 +34649,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Not capturable</t>
         </is>
@@ -34661,7 +34661,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>To confirm</t>
         </is>

</xml_diff>